<commit_message>
feat(F-NAR-019): TREE-AUT-034 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-034.xlsx
+++ b/stories/arbres/TREE-AUT-034.xlsx
@@ -4593,17 +4593,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Amir tend la corde le long du sillon du râteau. Le torchon s'y couche, en pente douce. Le manche, au mur, ne vole plus le fil. Un chemin d'ombre ! La coquille s'engage dessous, lente. La corde a trouvé mieux qu'un tas. Et le fer a trouvé le mur. L'herbe se relève où le râteau couchait.</t>
+          <t>Amir tend la corde le long de la trace du râteau. Le torchon s'y couche, en pente douce. Le manche, au mur, ne vole plus le fil. Un chemin d'ombre ! La coquille s'engage dessous, lente. La corde a trouvé mieux qu'un tas. Et le fer a trouvé le mur. L'herbe se relève où le râteau couchait.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir tend la &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; le long du sillon du râteau. Le torchon s'y couche, en pente douce. Le manche, au mur, ne vole plus le fil. Un chemin d'ombre ! La coquille s'engage dessous, lente. La corde a trouvé mieux qu'un tas. Et le fer a trouvé le mur. L'herbe se relève où le râteau couchait.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir tend la &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; le long de la trace du râteau. Le torchon s'y couche, en pente douce. Le manche, au mur, ne vole plus le fil. Un chemin d'ombre ! La coquille s'engage dessous, lente. La corde a trouvé mieux qu'un tas. Et le fer a trouvé le mur. L'herbe se relève où le râteau couchait.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Amir tend la &lt;emphasis&gt;corde&lt;/emphasis&gt; le long du sillon du râteau. Le torchon s'y couche, en pente douce. Le manche, au mur, ne vole plus le fil. Un chemin d'ombre ! La coquille s'engage dessous, lente. La corde a trouvé mieux qu'un tas. Et le fer a trouvé le mur. L'herbe se relève où le râteau couchait. [pause]</t>
+          <t>Amir tend la &lt;emphasis&gt;corde&lt;/emphasis&gt; le long de la trace du râteau. Le torchon s'y couche, en pente douce. Le manche, au mur, ne vole plus le fil. Un chemin d'ombre ! La coquille s'engage dessous, lente. La corde a trouvé mieux qu'un tas. Et le fer a trouvé le mur. L'herbe se relève où le râteau couchait. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>narrateur|Amir tend la corde le long du sillon du râteau.
+          <t>narrateur|Amir tend la corde le long de la trace du râteau.
 narrateur|Le torchon s'y couche, en pente douce.
 narrateur|Le manche, au mur, ne vole plus le fil.
 enfant-m|Un chemin d'ombre !
@@ -4776,17 +4776,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Amir suit du doigt le sillon vide. C'était le chemin du fer. Maintenant, c'est le chemin de la corde. L'herbe va se relever. Le manche au mur ne bouge plus. Sous le tissu, une virgule d'humidité brille.</t>
+          <t>Amir suit du doigt la trace vide. C'était le chemin du fer. Maintenant, c'est le chemin de la corde. L'herbe va se relever. Le manche au mur ne bouge plus. Sous le tissu, une petite trace mouillée brille.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir suit du doigt le sillon vide. C'était le chemin du fer. Maintenant, c'est le chemin de la &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt;. L'herbe va se relever. Le manche au mur ne bouge plus. Sous le tissu, une virgule d'humidité brille.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir suit du doigt la trace vide. C'était le chemin du fer. Maintenant, c'est le chemin de la &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt;. L'herbe va se relever. Le manche au mur ne bouge plus. Sous le tissu, une petite trace mouillée brille.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir suit du doigt le sillon vide. C'était le chemin du fer. Maintenant, c'est le chemin de la &lt;emphasis&gt;corde&lt;/emphasis&gt;. L'herbe va se relever. Le manche au mur ne bouge plus. Sous le tissu, une virgule d'humidité brille.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir suit du doigt la trace vide. C'était le chemin du fer. Maintenant, c'est le chemin de la &lt;emphasis&gt;corde&lt;/emphasis&gt;. L'herbe va se relever. Le manche au mur ne bouge plus. Sous le tissu, une petite trace mouillée brille.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -4924,12 +4924,12 @@
       </c>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>narrateur|Amir suit du doigt le sillon vide.
+          <t>narrateur|Amir suit du doigt la trace vide.
 papa|C'était le chemin du fer.
 enfant-m|Maintenant, c'est le chemin de la corde.
 maman|L'herbe va se relever.
 narrateur|Le manche au mur ne bouge plus.
-narrateur|Sous le tissu, une virgule d'humidité brille.</t>
+narrateur|Sous le tissu, une petite trace mouillée brille.</t>
         </is>
       </c>
       <c r="AX21" t="inlineStr">
@@ -8140,17 +8140,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Amir s'accroupit devant la porte de pinces. On frappe, avant d'entrer ? On n'entre pas, c'est chez lui. Tes bottes, elles, frappent le paillasson. Deux pinces font des sentinelles têtues. Au fond du bois, rien ne bouge, et c'est bien.</t>
+          <t>Amir s'accroupit devant la porte de pinces. On frappe, avant d'entrer ? On n'entre pas, c'est chez lui. Tes bottes, elles, frappent le paillasson. Deux pinces font des gardes bien droites. Au fond du bois, rien ne bouge, et c'est bien.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir s'accroupit devant la porte de &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt;. On frappe, avant d'entrer ? On n'entre pas, c'est chez lui. Tes bottes, elles, frappent le paillasson. Deux pinces font des sentinelles têtues. Au fond du bois, rien ne bouge, et c'est bien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir s'accroupit devant la porte de &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt;. On frappe, avant d'entrer ? On n'entre pas, c'est chez lui. Tes bottes, elles, frappent le paillasson. Deux pinces font des gardes bien droites. Au fond du bois, rien ne bouge, et c'est bien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir s'accroupit devant la porte de &lt;emphasis&gt;pinces&lt;/emphasis&gt;. On frappe, avant d'entrer ? On n'entre pas, c'est chez lui. Tes bottes, elles, frappent le paillasson. Deux pinces font des sentinelles têtues. Au fond du bois, rien ne bouge, et c'est bien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir s'accroupit devant la porte de &lt;emphasis&gt;pinces&lt;/emphasis&gt;. On frappe, avant d'entrer ? On n'entre pas, c'est chez lui. Tes bottes, elles, frappent le paillasson. Deux pinces font des gardes bien droites. Au fond du bois, rien ne bouge, et c'est bien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -8292,7 +8292,7 @@
 papa|On frappe, avant d'entrer ?
 enfant-m|On n'entre pas, c'est chez lui.
 maman|Tes bottes, elles, frappent le paillasson.
-narrateur|Deux pinces font des sentinelles têtues.
+narrateur|Deux pinces font des gardes bien droites.
 narrateur|Au fond du bois, rien ne bouge, et c'est bien.</t>
         </is>
       </c>
@@ -8693,17 +8693,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Amir glisse le seau dans l'ouverture de la caisse. Le bleu fait un sas avant le bois. Deux maisons, l'une dans l'autre ! L'escargot choisit d'abord le seau, plus frais. Le seau était vide, il servait à rien. Là, il sert à l'ombre. Une botte sèche au loin, oubliée du drame. Dans le bois, un silence rond.</t>
+          <t>Amir glisse le seau dans l'ouverture de la caisse. Le bleu fait une entrée avant le bois. Deux maisons, l'une dans l'autre ! L'escargot choisit d'abord le seau, plus frais. Le seau était vide, il servait à rien. Là, il sert à l'ombre. Une botte sèche au loin, oubliée du drame. Dans le bois, un silence rond.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir glisse le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; dans l'ouverture de la caisse. Le bleu fait un sas avant le bois. Deux maisons, l'une dans l'autre ! L'escargot choisit d'abord le seau, plus frais. Le seau était vide, il servait à rien. Là, il sert à l'ombre. Une botte sèche au loin, oubliée du drame. Dans le bois, un silence rond.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir glisse le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; dans l'ouverture de la caisse. Le bleu fait une entrée avant le bois. Deux maisons, l'une dans l'autre ! L'escargot choisit d'abord le seau, plus frais. Le seau était vide, il servait à rien. Là, il sert à l'ombre. Une botte sèche au loin, oubliée du drame. Dans le bois, un silence rond.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Amir glisse le &lt;emphasis&gt;seau&lt;/emphasis&gt; dans l'ouverture de la caisse. Le bleu fait un sas avant le bois. Deux maisons, l'une dans l'autre ! L'escargot choisit d'abord le seau, plus frais. Le seau était vide, il servait à rien. Là, il sert à l'ombre. Une botte sèche au loin, oubliée du drame. Dans le bois, un silence rond. [pause]</t>
+          <t>Amir glisse le &lt;emphasis&gt;seau&lt;/emphasis&gt; dans l'ouverture de la caisse. Le bleu fait une entrée avant le bois. Deux maisons, l'une dans l'autre ! L'escargot choisit d'abord le seau, plus frais. Le seau était vide, il servait à rien. Là, il sert à l'ombre. Une botte sèche au loin, oubliée du drame. Dans le bois, un silence rond. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -8838,7 +8838,7 @@
       <c r="AW42" t="inlineStr">
         <is>
           <t>narrateur|Amir glisse le seau dans l'ouverture de la caisse.
-narrateur|Le bleu fait un sas avant le bois.
+narrateur|Le bleu fait une entrée avant le bois.
 enfant-m|Deux maisons, l'une dans l'autre !
 narrateur|L'escargot choisit d'abord le seau, plus frais.
 papa|Le seau était vide, il servait à rien.
@@ -8876,17 +8876,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Amir aligne l'arrosoir, le seau, et la caisse du regard. Une famille de contenants ? Le seau pour entrer, la caisse pour dormir. Les bottes pour tes pieds, à la porte. Le bleu du sas capte un rond de ciel. Derrière, le bois reste nuit.</t>
+          <t>Amir aligne l'arrosoir, le seau, et la caisse du regard. L'arrosoir, le seau, et la caisse ? Le seau pour entrer, la caisse pour dormir. Les bottes pour tes pieds, à la porte. Le bleu de l'entrée capte un rond de ciel. Derrière, le bois reste nuit.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir aligne l'arrosoir, le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt;, et la caisse du regard. Une famille de contenants ? Le seau pour entrer, la caisse pour dormir. Les bottes pour tes pieds, à la porte. Le bleu du sas capte un rond de ciel. Derrière, le bois reste nuit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir aligne l'arrosoir, le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt;, et la caisse du regard. L'arrosoir, le seau, et la caisse ? Le seau pour entrer, la caisse pour dormir. Les bottes pour tes pieds, à la porte. Le bleu de l'entrée capte un rond de ciel. Derrière, le bois reste nuit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir aligne l'arrosoir, le &lt;emphasis&gt;seau&lt;/emphasis&gt;, et la caisse du regard. Une famille de contenants ? Le seau pour entrer, la caisse pour dormir. Les bottes pour tes pieds, à la porte. Le bleu du sas capte un rond de ciel. Derrière, le bois reste nuit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir aligne l'arrosoir, le &lt;emphasis&gt;seau&lt;/emphasis&gt;, et la caisse du regard. L'arrosoir, le seau, et la caisse ? Le seau pour entrer, la caisse pour dormir. Les bottes pour tes pieds, à la porte. Le bleu de l'entrée capte un rond de ciel. Derrière, le bois reste nuit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -9025,10 +9025,10 @@
       <c r="AW43" t="inlineStr">
         <is>
           <t>narrateur|Amir aligne l'arrosoir, le seau, et la caisse du regard.
-papa|Une famille de contenants ?
+papa|L'arrosoir, le seau, et la caisse ?
 enfant-m|Le seau pour entrer, la caisse pour dormir.
 maman|Les bottes pour tes pieds, à la porte.
-narrateur|Le bleu du sas capte un rond de ciel.
+narrateur|Le bleu de l'entrée capte un rond de ciel.
 narrateur|Derrière, le bois reste nuit.</t>
         </is>
       </c>
@@ -9447,17 +9447,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Amir plante les pinces de chaque côté de l'entrée. La caisse ouvre une bouche vers l'herbe. Le sillon du râteau passe à côté, vide. Pas de fer dans la porte. L'escargot s'engage, sans un bruit. Les pinces tiennent le rideau d'herbe. Le râteau, au mur, se tait. Un rai de soleil meurt sur le bois.</t>
+          <t>Amir plante les pinces de chaque côté de l'entrée. La caisse ouvre une bouche vers l'herbe. La trace du râteau passe à côté, vide. Pas de fer dans la porte. L'escargot s'engage, sans un bruit. Les pinces tiennent le rideau d'herbe. Le râteau, au mur, se tait. Un rayon de soleil s'arrête sur le bois.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir plante les &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt; de chaque côté de l'entrée. La caisse ouvre une bouche vers l'herbe. Le sillon du râteau passe à côté, vide. Pas de fer dans la porte. L'escargot s'engage, sans un bruit. Les pinces tiennent le rideau d'herbe. Le râteau, au mur, se tait. Un rai de soleil meurt sur le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir plante les &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt; de chaque côté de l'entrée. La caisse ouvre une bouche vers l'herbe. La trace du râteau passe à côté, vide. Pas de fer dans la porte. L'escargot s'engage, sans un bruit. Les pinces tiennent le rideau d'herbe. Le râteau, au mur, se tait. Un rayon de soleil s'arrête sur le bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Amir plante les &lt;emphasis&gt;pinces&lt;/emphasis&gt; de chaque côté de l'entrée. La caisse ouvre une bouche vers l'herbe. Le sillon du râteau passe à côté, vide. Pas de fer dans la porte. L'escargot s'engage, sans un bruit. Les pinces tiennent le rideau d'herbe. Le râteau, au mur, se tait. Un rai de soleil meurt sur le bois. [pause]</t>
+          <t>Amir plante les &lt;emphasis&gt;pinces&lt;/emphasis&gt; de chaque côté de l'entrée. La caisse ouvre une bouche vers l'herbe. La trace du râteau passe à côté, vide. Pas de fer dans la porte. L'escargot s'engage, sans un bruit. Les pinces tiennent le rideau d'herbe. Le râteau, au mur, se tait. Un rayon de soleil s'arrête sur le bois. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9593,12 +9593,12 @@
         <is>
           <t>narrateur|Amir plante les pinces de chaque côté de l'entrée.
 narrateur|La caisse ouvre une bouche vers l'herbe.
-narrateur|Le sillon du râteau passe à côté, vide.
+narrateur|La trace du râteau passe à côté, vide.
 enfant-m|Pas de fer dans la porte.
 narrateur|L'escargot s'engage, sans un bruit.
 maman|Les pinces tiennent le rideau d'herbe.
 papa|Le râteau, au mur, se tait.
-narrateur|Un rai de soleil meurt sur le bois.</t>
+narrateur|Un rayon de soleil s'arrête sur le bois.</t>
         </is>
       </c>
       <c r="AX46" t="inlineStr">
@@ -9630,17 +9630,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Amir écarte l'herbe à l'entrée, sans la casser. Les pinces tiennent ça ? Oui, pas de fer dans la porte. Le râteau a son mur, c'est mieux. Un rai meurt sur le seuil. Dedans, la caisse sent l'humide et le calme.</t>
+          <t>Amir écarte l'herbe à l'entrée, sans la casser. Les pinces tiennent ça ? Oui, pas de fer dans la porte. Le râteau a son mur, c'est mieux. Un rayon s'arrête sur le seuil. Dedans, la caisse sent l'humide et le calme.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir écarte l'herbe à l'entrée, sans la casser. Les &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt; tiennent ça ? Oui, pas de fer dans la porte. Le râteau a son mur, c'est mieux. Un rai meurt sur le seuil. Dedans, la caisse sent l'humide et le calme.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir écarte l'herbe à l'entrée, sans la casser. Les &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt; tiennent ça ? Oui, pas de fer dans la porte. Le râteau a son mur, c'est mieux. Un rayon s'arrête sur le seuil. Dedans, la caisse sent l'humide et le calme.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir écarte l'herbe à l'entrée, sans la casser. Les &lt;emphasis&gt;pinces&lt;/emphasis&gt; tiennent ça ? Oui, pas de fer dans la porte. Le râteau a son mur, c'est mieux. Un rai meurt sur le seuil. Dedans, la caisse sent l'humide et le calme.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir écarte l'herbe à l'entrée, sans la casser. Les &lt;emphasis&gt;pinces&lt;/emphasis&gt; tiennent ça ? Oui, pas de fer dans la porte. Le râteau a son mur, c'est mieux. Un rayon s'arrête sur le seuil. Dedans, la caisse sent l'humide et le calme.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9782,7 +9782,7 @@
 papa|Les pinces tiennent ça ?
 enfant-m|Oui, pas de fer dans la porte.
 maman|Le râteau a son mur, c'est mieux.
-narrateur|Un rai meurt sur le seuil.
+narrateur|Un rayon s'arrête sur le seuil.
 narrateur|Dedans, la caisse sent l'humide et le calme.</t>
         </is>
       </c>
@@ -9815,17 +9815,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Amir attache la corde au rebord de la caisse. Il l'ancre dans le sillon du râteau. La grotte ne peut plus basculer. Elle est amarrée ! L'escargot entre, rassuré par l'immobilité. La corde a gagné contre le manche. Le fer dort au mur. Le bois ne tremble plus.</t>
+          <t>Amir attache la corde au rebord de la caisse. Il la fixe dans la trace du râteau. La grotte ne peut plus basculer. Elle est attachée ! L'escargot entre, rassuré : plus rien ne bouge. La corde a gagné contre le manche. Le fer dort au mur. Le bois ne tremble plus.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir attache la &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; au rebord de la caisse. Il l'ancre dans le sillon du râteau. La grotte ne peut plus basculer. Elle est amarrée ! L'escargot entre, rassuré par l'immobilité. La corde a gagné contre le manche. Le fer dort au mur. Le bois ne tremble plus.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir attache la &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; au rebord de la caisse. Il la fixe dans la trace du râteau. La grotte ne peut plus basculer. Elle est attachée ! L'escargot entre, rassuré : plus rien ne bouge. La corde a gagné contre le manche. Le fer dort au mur. Le bois ne tremble plus.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Amir attache la &lt;emphasis&gt;corde&lt;/emphasis&gt; au rebord de la caisse. Il l'ancre dans le sillon du râteau. La grotte ne peut plus basculer. Elle est amarrée ! L'escargot entre, rassuré par l'immobilité. La corde a gagné contre le manche. Le fer dort au mur. Le bois ne tremble plus. [pause]</t>
+          <t>Amir attache la &lt;emphasis&gt;corde&lt;/emphasis&gt; au rebord de la caisse. Il la fixe dans la trace du râteau. La grotte ne peut plus basculer. Elle est attachée ! L'escargot entre, rassuré : plus rien ne bouge. La corde a gagné contre le manche. Le fer dort au mur. Le bois ne tremble plus. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -9960,10 +9960,10 @@
       <c r="AW48" t="inlineStr">
         <is>
           <t>narrateur|Amir attache la corde au rebord de la caisse.
-narrateur|Il l'ancre dans le sillon du râteau.
+narrateur|Il la fixe dans la trace du râteau.
 narrateur|La grotte ne peut plus basculer.
-enfant-m|Elle est amarrée !
-narrateur|L'escargot entre, rassuré par l'immobilité.
+enfant-m|Elle est attachée !
+narrateur|L'escargot entre, rassuré : plus rien ne bouge.
 papa|La corde a gagné contre le manche.
 maman|Le fer dort au mur.
 narrateur|Le bois ne tremble plus.</t>
@@ -9998,17 +9998,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Amir appuie sur la caisse : rien ne bascule. Amarrée pour de bon ? La corde a gagné contre le manche. Le fer dort, le bois veille. Le sillon du râteau sert d'ancre, à présent. L'escargot n'entend plus le clac du fer.</t>
+          <t>Amir appuie sur la caisse : rien ne bascule. Attachée pour de bon ? La corde a gagné contre le manche. Le fer dort, le bois veille. La trace du râteau sert à tenir, maintenant. L'escargot n'entend plus le clac du fer.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir appuie sur la caisse : rien ne bascule. Amarrée pour de bon ? La &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; a gagné contre le manche. Le fer dort, le bois veille. Le sillon du râteau sert d'ancre, à présent. L'escargot n'entend plus le clac du fer.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir appuie sur la caisse : rien ne bascule. Attachée pour de bon ? La &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; a gagné contre le manche. Le fer dort, le bois veille. La trace du râteau sert à tenir, maintenant. L'escargot n'entend plus le clac du fer.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir appuie sur la caisse : rien ne bascule. Amarrée pour de bon ? La &lt;emphasis&gt;corde&lt;/emphasis&gt; a gagné contre le manche. Le fer dort, le bois veille. Le sillon du râteau sert d'ancre, à présent. L'escargot n'entend plus le clac du fer.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir appuie sur la caisse : rien ne bascule. Attachée pour de bon ? La &lt;emphasis&gt;corde&lt;/emphasis&gt; a gagné contre le manche. Le fer dort, le bois veille. La trace du râteau sert à tenir, maintenant. L'escargot n'entend plus le clac du fer.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10147,10 +10147,10 @@
       <c r="AW49" t="inlineStr">
         <is>
           <t>narrateur|Amir appuie sur la caisse : rien ne bascule.
-papa|Amarrée pour de bon ?
+papa|Attachée pour de bon ?
 enfant-m|La corde a gagné contre le manche.
 maman|Le fer dort, le bois veille.
-narrateur|Le sillon du râteau sert d'ancre, à présent.
+narrateur|La trace du râteau sert à tenir, maintenant.
 narrateur|L'escargot n'entend plus le clac du fer.</t>
         </is>
       </c>
@@ -10936,17 +10936,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Amir pince un coin de chiffon à l'entrée de la caisse. Le chiffon sent la prune, un peu. Un rideau sucré ! L'escargot soulève le tissu, puis passe. Les pinces tiennent le parfum dehors. Le panier, sur le banc, garde le reste. Une tache violette sèche au soleil du banc. Dans la caisse, l'air reste neutre.</t>
+          <t>Amir pince un coin de chiffon à l'entrée de la caisse. Le chiffon sent la prune, un peu. Un rideau sucré ! L'escargot soulève le tissu, puis passe. Les pinces tiennent le parfum dehors. Le panier, sur le banc, garde le reste. Une tache violette sèche au soleil du banc. Dans la caisse, l'air n'a plus de fruit.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir pince un coin de chiffon à l'entrée de la caisse. Le chiffon sent la prune, un peu. Un rideau sucré ! L'escargot soulève le tissu, puis passe. Les &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt; tiennent le parfum dehors. Le panier, sur le banc, garde le reste. Une tache violette sèche au soleil du banc. Dans la caisse, l'air reste neutre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir pince un coin de chiffon à l'entrée de la caisse. Le chiffon sent la prune, un peu. Un rideau sucré ! L'escargot soulève le tissu, puis passe. Les &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt; tiennent le parfum dehors. Le panier, sur le banc, garde le reste. Une tache violette sèche au soleil du banc. Dans la caisse, l'air n'a plus de fruit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Amir pince un coin de chiffon à l'entrée de la caisse. Le chiffon sent la prune, un peu. Un rideau sucré ! L'escargot soulève le tissu, puis passe. Les &lt;emphasis&gt;pinces&lt;/emphasis&gt; tiennent le parfum dehors. Le panier, sur le banc, garde le reste. Une tache violette sèche au soleil du banc. Dans la caisse, l'air reste neutre. [pause]</t>
+          <t>Amir pince un coin de chiffon à l'entrée de la caisse. Le chiffon sent la prune, un peu. Un rideau sucré ! L'escargot soulève le tissu, puis passe. Les &lt;emphasis&gt;pinces&lt;/emphasis&gt; tiennent le parfum dehors. Le panier, sur le banc, garde le reste. Une tache violette sèche au soleil du banc. Dans la caisse, l'air n'a plus de fruit. [pause]</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -11087,7 +11087,7 @@
 papa|Les pinces tiennent le parfum dehors.
 maman|Le panier, sur le banc, garde le reste.
 narrateur|Une tache violette sèche au soleil du banc.
-narrateur|Dans la caisse, l'air reste neutre.</t>
+narrateur|Dans la caisse, l'air n'a plus de fruit.</t>
         </is>
       </c>
       <c r="AX54" t="inlineStr">
@@ -11119,17 +11119,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Amir lève le rideau de chiffon, un millimètre. On dérange ? Non, je vérifie le parfum. Le sucre est resté sur le banc. Une tache violette sèche, loin de la caisse. Derrière le chiffon, l'air est plat, sans fruit.</t>
+          <t>Amir lève le rideau de chiffon, très peu. On dérange ? Non, je vérifie le parfum. Le sucre est resté sur le banc. Une tache violette sèche, loin de la caisse. Derrière le chiffon, l'air est plat, sans fruit.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir lève le rideau de chiffon, un millimètre. On dérange ? Non, je vérifie le parfum. Le sucre est resté sur le banc. Une tache violette sèche, loin de la caisse. Derrière le chiffon, l'air est plat, sans fruit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir lève le rideau de chiffon, très peu. On dérange ? Non, je vérifie le parfum. Le sucre est resté sur le banc. Une tache violette sèche, loin de la caisse. Derrière le chiffon, l'air est plat, sans fruit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir lève le rideau de chiffon, un millimètre. On dérange ? Non, je vérifie le parfum. Le sucre est resté sur le banc. Une tache violette sèche, loin de la caisse. Derrière le chiffon, l'air est plat, sans fruit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir lève le rideau de chiffon, très peu. On dérange ? Non, je vérifie le parfum. Le sucre est resté sur le banc. Une tache violette sèche, loin de la caisse. Derrière le chiffon, l'air est plat, sans fruit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11267,7 +11267,7 @@
       </c>
       <c r="AW55" t="inlineStr">
         <is>
-          <t>narrateur|Amir lève le rideau de chiffon, un millimètre.
+          <t>narrateur|Amir lève le rideau de chiffon, très peu.
 papa|On dérange ?
 enfant-m|Non, je vérifie le parfum.
 maman|Le sucre est resté sur le banc.
@@ -11672,17 +11672,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Amir pose le seau en sentinelle devant la caisse. Le bleu sépare le bois du banc aux prunes. Personne ne roule dessus. L'escargot entre par le côté, loin du fruit. Le seau fait le garde. Les prunes font la confiture, plus tard. Une odeur sucrée s'arrête au bleu. Au fond de la caisse, la terre sent l'humide.</t>
+          <t>Amir pose le seau en garde devant la caisse. Le bleu sépare le bois du banc aux prunes. Personne ne roule dessus. L'escargot entre par le côté, loin du fruit. Le seau fait le garde. Les prunes font la confiture, plus tard. Une odeur sucrée s'arrête au bleu. Au fond de la caisse, la terre sent l'humide.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir pose le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; en sentinelle devant la caisse. Le bleu sépare le bois du banc aux prunes. Personne ne roule dessus. L'escargot entre par le côté, loin du fruit. Le seau fait le garde. Les prunes font la confiture, plus tard. Une odeur sucrée s'arrête au bleu. Au fond de la caisse, la terre sent l'humide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir pose le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; en garde devant la caisse. Le bleu sépare le bois du banc aux prunes. Personne ne roule dessus. L'escargot entre par le côté, loin du fruit. Le seau fait le garde. Les prunes font la confiture, plus tard. Une odeur sucrée s'arrête au bleu. Au fond de la caisse, la terre sent l'humide.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Amir pose le &lt;emphasis&gt;seau&lt;/emphasis&gt; en sentinelle devant la caisse. Le bleu sépare le bois du banc aux prunes. Personne ne roule dessus. L'escargot entre par le côté, loin du fruit. Le seau fait le garde. Les prunes font la confiture, plus tard. Une odeur sucrée s'arrête au bleu. Au fond de la caisse, la terre sent l'humide. [pause]</t>
+          <t>Amir pose le &lt;emphasis&gt;seau&lt;/emphasis&gt; en garde devant la caisse. Le bleu sépare le bois du banc aux prunes. Personne ne roule dessus. L'escargot entre par le côté, loin du fruit. Le seau fait le garde. Les prunes font la confiture, plus tard. Une odeur sucrée s'arrête au bleu. Au fond de la caisse, la terre sent l'humide. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11816,7 +11816,7 @@
       </c>
       <c r="AW58" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose le seau en sentinelle devant la caisse.
+          <t>narrateur|Amir pose le seau en garde devant la caisse.
 narrateur|Le bleu sépare le bois du banc aux prunes.
 enfant-m|Personne ne roule dessus.
 narrateur|L'escargot entre par le côté, loin du fruit.
@@ -11855,17 +11855,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Amir salue le seau-sentinelle d'un petit tapotement. Il laisse passer qui ? Lui, pas les prunes. La confiture attendra le soir. L'odeur sucrée s'arrête net au bleu. Au fond de la caisse, l'humide a gagné.</t>
+          <t>Amir salue le seau qui garde, d'un petit coup. Il laisse passer qui ? Lui, pas les prunes. La confiture attendra le soir. L'odeur sucrée s'arrête net au bleu. Au fond de la caisse, l'humide a gagné.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir salue le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt;-sentinelle d'un petit tapotement. Il laisse passer qui ? Lui, pas les prunes. La confiture attendra le soir. L'odeur sucrée s'arrête net au bleu. Au fond de la caisse, l'humide a gagné.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir salue le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; qui garde, d'un petit coup. Il laisse passer qui ? Lui, pas les prunes. La confiture attendra le soir. L'odeur sucrée s'arrête net au bleu. Au fond de la caisse, l'humide a gagné.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir salue le &lt;emphasis&gt;seau&lt;/emphasis&gt;-sentinelle d'un petit tapotement. Il laisse passer qui ? Lui, pas les prunes. La confiture attendra le soir. L'odeur sucrée s'arrête net au bleu. Au fond de la caisse, l'humide a gagné.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir salue le &lt;emphasis&gt;seau&lt;/emphasis&gt; qui garde, d'un petit coup. Il laisse passer qui ? Lui, pas les prunes. La confiture attendra le soir. L'odeur sucrée s'arrête net au bleu. Au fond de la caisse, l'humide a gagné.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12003,7 +12003,7 @@
       </c>
       <c r="AW59" t="inlineStr">
         <is>
-          <t>narrateur|Amir salue le seau-sentinelle d'un petit tapotement.
+          <t>narrateur|Amir salue le seau qui garde, d'un petit coup.
 papa|Il laisse passer qui ?
 enfant-m|Lui, pas les prunes.
 maman|La confiture attendra le soir.
@@ -13178,17 +13178,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Amir plante les pinces autour du creux mouillé. Elles tiennent un lambeau de torchon, juste assez. Un puits avec un chapeau ! L'escargot redescend vers l'eau, à l'ombre. Les pinces n'ont pas mouillé, elles. Tes bottes non plus, à présent. Le creux brille, petit miroir. Une corne y boit, ou presque.</t>
+          <t>Amir plante les pinces autour du creux mouillé. Elles tiennent un bout de torchon, juste assez. Un puits avec un chapeau ! L'escargot redescend vers l'eau, à l'ombre. Les pinces n'ont pas mouillé, elles. Tes bottes non plus, maintenant. Le creux brille, petit miroir. Une corne y boit, ou presque.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir plante les &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt; autour du creux mouillé. Elles tiennent un lambeau de torchon, juste assez. Un puits avec un chapeau ! L'escargot redescend vers l'eau, à l'ombre. Les pinces n'ont pas mouillé, elles. Tes bottes non plus, à présent. Le creux brille, petit miroir. Une corne y boit, ou presque.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir plante les &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt; autour du creux mouillé. Elles tiennent un bout de torchon, juste assez. Un puits avec un chapeau ! L'escargot redescend vers l'eau, à l'ombre. Les pinces n'ont pas mouillé, elles. Tes bottes non plus, maintenant. Le creux brille, petit miroir. Une corne y boit, ou presque.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Amir plante les &lt;emphasis&gt;pinces&lt;/emphasis&gt; autour du creux mouillé. Elles tiennent un lambeau de torchon, juste assez. Un puits avec un chapeau ! L'escargot redescend vers l'eau, à l'ombre. Les pinces n'ont pas mouillé, elles. Tes bottes non plus, à présent. Le creux brille, petit miroir. Une corne y boit, ou presque. [pause]</t>
+          <t>Amir plante les &lt;emphasis&gt;pinces&lt;/emphasis&gt; autour du creux mouillé. Elles tiennent un bout de torchon, juste assez. Un puits avec un chapeau ! L'escargot redescend vers l'eau, à l'ombre. Les pinces n'ont pas mouillé, elles. Tes bottes non plus, maintenant. Le creux brille, petit miroir. Une corne y boit, ou presque. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13323,11 +13323,11 @@
       <c r="AW66" t="inlineStr">
         <is>
           <t>narrateur|Amir plante les pinces autour du creux mouillé.
-narrateur|Elles tiennent un lambeau de torchon, juste assez.
+narrateur|Elles tiennent un bout de torchon, juste assez.
 enfant-m|Un puits avec un chapeau !
 narrateur|L'escargot redescend vers l'eau, à l'ombre.
 papa|Les pinces n'ont pas mouillé, elles.
-maman|Tes bottes non plus, à présent.
+maman|Tes bottes non plus, maintenant.
 narrateur|Le creux brille, petit miroir.
 narrateur|Une corne y boit, ou presque.</t>
         </is>
@@ -13546,17 +13546,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Amir tend la corde au-dessus du filet d'eau. Un coin de tissu y pend, comme un auvent. L'eau reste à lui. L'escargot longe le frais, sous le tissu. La corde fait le pont, sans bottes dessous. Au paillasson, le cuir sèche. Le filet ne part plus vers la porte. Il tourne autour de la feuille.</t>
+          <t>Amir tend la corde au-dessus du filet d'eau. Un coin de tissu y pend, comme un petit toit. L'eau reste à lui. L'escargot longe le frais, sous le tissu. La corde fait le pont, sans bottes dessous. Au paillasson, le cuir sèche. Le filet ne part plus vers la porte. Il tourne autour de la feuille.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir tend la &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; au-dessus du filet d'eau. Un coin de tissu y pend, comme un auvent. L'eau reste à lui. L'escargot longe le frais, sous le tissu. La corde fait le pont, sans bottes dessous. Au paillasson, le cuir sèche. Le filet ne part plus vers la porte. Il tourne autour de la feuille.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir tend la &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; au-dessus du filet d'eau. Un coin de tissu y pend, comme un petit toit. L'eau reste à lui. L'escargot longe le frais, sous le tissu. La corde fait le pont, sans bottes dessous. Au paillasson, le cuir sèche. Le filet ne part plus vers la porte. Il tourne autour de la feuille.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Amir tend la &lt;emphasis&gt;corde&lt;/emphasis&gt; au-dessus du filet d'eau. Un coin de tissu y pend, comme un auvent. L'eau reste à lui. L'escargot longe le frais, sous le tissu. La corde fait le pont, sans bottes dessous. Au paillasson, le cuir sèche. Le filet ne part plus vers la porte. Il tourne autour de la feuille. [pause]</t>
+          <t>Amir tend la &lt;emphasis&gt;corde&lt;/emphasis&gt; au-dessus du filet d'eau. Un coin de tissu y pend, comme un petit toit. L'eau reste à lui. L'escargot longe le frais, sous le tissu. La corde fait le pont, sans bottes dessous. Au paillasson, le cuir sèche. Le filet ne part plus vers la porte. Il tourne autour de la feuille. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13691,7 +13691,7 @@
       <c r="AW68" t="inlineStr">
         <is>
           <t>narrateur|Amir tend la corde au-dessus du filet d'eau.
-narrateur|Un coin de tissu y pend, comme un auvent.
+narrateur|Un coin de tissu y pend, comme un petit toit.
 enfant-m|L'eau reste à lui.
 narrateur|L'escargot longe le frais, sous le tissu.
 maman|La corde fait le pont, sans bottes dessous.
@@ -13729,17 +13729,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Amir suit l'eau du regard : elle tourne, elle reste. Plus de fuite vers la porte ? La corde a fermé le chemin des bottes. Le cuir peut sécher. Un auvent de tissu tremble, très peu. Autour de la feuille, le filet fait un collier.</t>
+          <t>Amir suit l'eau du regard : elle tourne, elle reste. Plus de fuite vers la porte ? La corde a fermé le chemin des bottes. Le cuir peut sécher. Un petit toit de tissu tremble, très peu. Autour de la feuille, le filet fait un collier.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir suit l'eau du regard : elle tourne, elle reste. Plus de fuite vers la porte ? La &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; a fermé le chemin des bottes. Le cuir peut sécher. Un auvent de tissu tremble, très peu. Autour de la feuille, le filet fait un collier.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir suit l'eau du regard : elle tourne, elle reste. Plus de fuite vers la porte ? La &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; a fermé le chemin des bottes. Le cuir peut sécher. Un petit toit de tissu tremble, très peu. Autour de la feuille, le filet fait un collier.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir suit l'eau du regard : elle tourne, elle reste. Plus de fuite vers la porte ? La &lt;emphasis&gt;corde&lt;/emphasis&gt; a fermé le chemin des bottes. Le cuir peut sécher. Un auvent de tissu tremble, très peu. Autour de la feuille, le filet fait un collier.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir suit l'eau du regard : elle tourne, elle reste. Plus de fuite vers la porte ? La &lt;emphasis&gt;corde&lt;/emphasis&gt; a fermé le chemin des bottes. Le cuir peut sécher. Un petit toit de tissu tremble, très peu. Autour de la feuille, le filet fait un collier.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -13881,7 +13881,7 @@
 papa|Plus de fuite vers la porte ?
 enfant-m|La corde a fermé le chemin des bottes.
 maman|Le cuir peut sécher.
-narrateur|Un auvent de tissu tremble, très peu.
+narrateur|Un petit toit de tissu tremble, très peu.
 narrateur|Autour de la feuille, le filet fait un collier.</t>
         </is>
       </c>
@@ -14667,17 +14667,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Amir pince un toit au-dessus du creux, hors du sillon. L'eau ne suit plus le fer. Elle reste en rond. L'escargot s'installe au bord, à l'ombre des pinces. Les pinces font un cercle, pas un fleuve. Le râteau, au mur, n'oriente plus l'eau. Une dent sèche capte la lumière, loin. Près de la feuille, tout est mat.</t>
+          <t>Amir pince un toit au-dessus du creux, hors de la trace. L'eau ne suit plus le fer. Elle reste en rond. L'escargot s'installe au bord, à l'ombre des pinces. Les pinces font un cercle, pas un fleuve. Le râteau, au mur, ne pousse plus l'eau. Une dent sèche capte la lumière, loin. Près de la feuille, tout est mat.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir pince un toit au-dessus du creux, hors du sillon. L'eau ne suit plus le fer. Elle reste en rond. L'escargot s'installe au bord, à l'ombre des &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt;. Les pinces font un cercle, pas un fleuve. Le râteau, au mur, n'oriente plus l'eau. Une dent sèche capte la lumière, loin. Près de la feuille, tout est mat.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir pince un toit au-dessus du creux, hors de la trace. L'eau ne suit plus le fer. Elle reste en rond. L'escargot s'installe au bord, à l'ombre des &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt;. Les pinces font un cercle, pas un fleuve. Le râteau, au mur, ne pousse plus l'eau. Une dent sèche capte la lumière, loin. Près de la feuille, tout est mat.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Amir pince un toit au-dessus du creux, hors du sillon. L'eau ne suit plus le fer. Elle reste en rond. L'escargot s'installe au bord, à l'ombre des &lt;emphasis&gt;pinces&lt;/emphasis&gt;. Les pinces font un cercle, pas un fleuve. Le râteau, au mur, n'oriente plus l'eau. Une dent sèche capte la lumière, loin. Près de la feuille, tout est mat. [pause]</t>
+          <t>Amir pince un toit au-dessus du creux, hors de la trace. L'eau ne suit plus le fer. Elle reste en rond. L'escargot s'installe au bord, à l'ombre des &lt;emphasis&gt;pinces&lt;/emphasis&gt;. Les pinces font un cercle, pas un fleuve. Le râteau, au mur, ne pousse plus l'eau. Une dent sèche capte la lumière, loin. Près de la feuille, tout est mat. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -14811,12 +14811,12 @@
       </c>
       <c r="AW74" t="inlineStr">
         <is>
-          <t>narrateur|Amir pince un toit au-dessus du creux, hors du sillon.
+          <t>narrateur|Amir pince un toit au-dessus du creux, hors de la trace.
 narrateur|L'eau ne suit plus le fer.
 enfant-m|Elle reste en rond.
 narrateur|L'escargot s'installe au bord, à l'ombre des pinces.
 maman|Les pinces font un cercle, pas un fleuve.
-papa|Le râteau, au mur, n'oriente plus l'eau.
+papa|Le râteau, au mur, ne pousse plus l'eau.
 narrateur|Une dent sèche capte la lumière, loin.
 narrateur|Près de la feuille, tout est mat.</t>
         </is>
@@ -14850,17 +14850,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Amir compare le cercle des pinces et le sillon vide. Rond contre ligne ? Le rond est pour lui, la ligne est finie. Le râteau n'écrit plus sur l'eau. Une dent sèche, au mur, garde un éclat. Près de la feuille, l'eau est mate, ronde, sage.</t>
+          <t>Amir compare le cercle des pinces et la trace vide. Rond contre ligne ? Le rond est pour lui, la ligne est finie. Le râteau n'écrit plus sur l'eau. Une dent sèche, au mur, garde un éclat. Près de la feuille, l'eau est mate, ronde, sage.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir compare le cercle des &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt; et le sillon vide. Rond contre ligne ? Le rond est pour lui, la ligne est finie. Le râteau n'écrit plus sur l'eau. Une dent sèche, au mur, garde un éclat. Près de la feuille, l'eau est mate, ronde, sage.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir compare le cercle des &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt; et la trace vide. Rond contre ligne ? Le rond est pour lui, la ligne est finie. Le râteau n'écrit plus sur l'eau. Une dent sèche, au mur, garde un éclat. Près de la feuille, l'eau est mate, ronde, sage.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir compare le cercle des &lt;emphasis&gt;pinces&lt;/emphasis&gt; et le sillon vide. Rond contre ligne ? Le rond est pour lui, la ligne est finie. Le râteau n'écrit plus sur l'eau. Une dent sèche, au mur, garde un éclat. Près de la feuille, l'eau est mate, ronde, sage.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir compare le cercle des &lt;emphasis&gt;pinces&lt;/emphasis&gt; et la trace vide. Rond contre ligne ? Le rond est pour lui, la ligne est finie. Le râteau n'écrit plus sur l'eau. Une dent sèche, au mur, garde un éclat. Près de la feuille, l'eau est mate, ronde, sage.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -14998,7 +14998,7 @@
       </c>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>narrateur|Amir compare le cercle des pinces et le sillon vide.
+          <t>narrateur|Amir compare le cercle des pinces et la trace vide.
 papa|Rond contre ligne ?
 enfant-m|Le rond est pour lui, la ligne est finie.
 maman|Le râteau n'écrit plus sur l'eau.
@@ -15035,17 +15035,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Amir barre le sillon avec la corde, à plat. L'eau s'arrête et forme une mare. J'ai fermé la rivière ! L'escargot contourne la mare, sous un lambeau tendu. La corde a battu le manche. Le mur garde le fer. La mare tremble, puis se calme. Deux cornes s'y reflètent, un instant.</t>
+          <t>Amir barre la trace avec la corde, à plat. L'eau s'arrête et forme une mare. J'ai fermé la rivière ! L'escargot contourne la mare, sous un bout tendu. La corde a battu le manche. Le mur garde le fer. La mare tremble, puis se calme. Deux cornes s'y reflètent, un instant.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir barre le sillon avec la &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt;, à plat. L'eau s'arrête et forme une mare. J'ai fermé la rivière ! L'escargot contourne la mare, sous un lambeau tendu. La corde a battu le manche. Le mur garde le fer. La mare tremble, puis se calme. Deux cornes s'y reflètent, un instant.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir barre la trace avec la &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt;, à plat. L'eau s'arrête et forme une mare. J'ai fermé la rivière ! L'escargot contourne la mare, sous un bout tendu. La corde a battu le manche. Le mur garde le fer. La mare tremble, puis se calme. Deux cornes s'y reflètent, un instant.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Amir barre le sillon avec la &lt;emphasis&gt;corde&lt;/emphasis&gt;, à plat. L'eau s'arrête et forme une mare. J'ai fermé la rivière ! L'escargot contourne la mare, sous un lambeau tendu. La corde a battu le manche. Le mur garde le fer. La mare tremble, puis se calme. Deux cornes s'y reflètent, un instant. [pause]</t>
+          <t>Amir barre la trace avec la &lt;emphasis&gt;corde&lt;/emphasis&gt;, à plat. L'eau s'arrête et forme une mare. J'ai fermé la rivière ! L'escargot contourne la mare, sous un bout tendu. La corde a battu le manche. Le mur garde le fer. La mare tremble, puis se calme. Deux cornes s'y reflètent, un instant. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15179,10 +15179,10 @@
       </c>
       <c r="AW76" t="inlineStr">
         <is>
-          <t>narrateur|Amir barre le sillon avec la corde, à plat.
+          <t>narrateur|Amir barre la trace avec la corde, à plat.
 narrateur|L'eau s'arrête et forme une mare.
 enfant-m|J'ai fermé la rivière !
-narrateur|L'escargot contourne la mare, sous un lambeau tendu.
+narrateur|L'escargot contourne la mare, sous un bout tendu.
 papa|La corde a battu le manche.
 maman|Le mur garde le fer.
 narrateur|La mare tremble, puis se calme.
@@ -15218,17 +15218,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Amir se voit, un instant, dans la mare. Deux cornes aussi ? Oui, il est là, sous le lambeau. La corde a battu le fleuve du manche. La mare se calme, sans ride. Au mur, le fer n'oriente plus rien.</t>
+          <t>Amir se voit, un instant, dans la mare. Deux cornes aussi ? Oui, il est là, sous le tissu. La corde a battu le fleuve du manche. La mare se calme, sans ride. Au mur, le fer ne pousse plus l'eau.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir se voit, un instant, dans la mare. Deux cornes aussi ? Oui, il est là, sous le lambeau. La &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; a battu le fleuve du manche. La mare se calme, sans ride. Au mur, le fer n'oriente plus rien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir se voit, un instant, dans la mare. Deux cornes aussi ? Oui, il est là, sous le tissu. La &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; a battu le fleuve du manche. La mare se calme, sans ride. Au mur, le fer ne pousse plus l'eau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir se voit, un instant, dans la mare. Deux cornes aussi ? Oui, il est là, sous le lambeau. La &lt;emphasis&gt;corde&lt;/emphasis&gt; a battu le fleuve du manche. La mare se calme, sans ride. Au mur, le fer n'oriente plus rien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir se voit, un instant, dans la mare. Deux cornes aussi ? Oui, il est là, sous le tissu. La &lt;emphasis&gt;corde&lt;/emphasis&gt; a battu le fleuve du manche. La mare se calme, sans ride. Au mur, le fer ne pousse plus l'eau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -15368,10 +15368,10 @@
         <is>
           <t>narrateur|Amir se voit, un instant, dans la mare.
 papa|Deux cornes aussi ?
-enfant-m|Oui, il est là, sous le lambeau.
+enfant-m|Oui, il est là, sous le tissu.
 maman|La corde a battu le fleuve du manche.
 narrateur|La mare se calme, sans ride.
-narrateur|Au mur, le fer n'oriente plus rien.</t>
+narrateur|Au mur, le fer ne pousse plus l'eau.</t>
         </is>
       </c>
       <c r="AX77" t="inlineStr">
@@ -15403,17 +15403,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Amir pose le seau en travers du sillon mort. L'eau s'y rassemble, fraîche. Un réservoir pour lui. L'escargot gravit le bord humide, puis s'abrite. Le seau capte ce que le râteau répandait. Échange réussi. Une goutte tombe dedans, ploc. Au mur, le fer reste sec.</t>
+          <t>Amir pose le seau en travers de la trace vide. L'eau s'y rassemble, fraîche. Un réservoir pour lui. L'escargot gravit le bord humide, puis s'abrite. Le seau capte ce que le râteau répandait. Échange réussi. Une goutte tombe dedans, ploc. Au mur, le fer reste sec.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir pose le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; en travers du sillon mort. L'eau s'y rassemble, fraîche. Un réservoir pour lui. L'escargot gravit le bord humide, puis s'abrite. Le seau capte ce que le râteau répandait. Échange réussi. Une goutte tombe dedans, ploc. Au mur, le fer reste sec.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir pose le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; en travers de la trace vide. L'eau s'y rassemble, fraîche. Un réservoir pour lui. L'escargot gravit le bord humide, puis s'abrite. Le seau capte ce que le râteau répandait. Échange réussi. Une goutte tombe dedans, ploc. Au mur, le fer reste sec.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Amir pose le &lt;emphasis&gt;seau&lt;/emphasis&gt; en travers du sillon mort. L'eau s'y rassemble, fraîche. Un réservoir pour lui. L'escargot gravit le bord humide, puis s'abrite. Le seau capte ce que le râteau répandait. Échange réussi. Une goutte tombe dedans, ploc. Au mur, le fer reste sec. [pause]</t>
+          <t>Amir pose le &lt;emphasis&gt;seau&lt;/emphasis&gt; en travers de la trace vide. L'eau s'y rassemble, fraîche. Un réservoir pour lui. L'escargot gravit le bord humide, puis s'abrite. Le seau capte ce que le râteau répandait. Échange réussi. Une goutte tombe dedans, ploc. Au mur, le fer reste sec. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -15547,7 +15547,7 @@
       </c>
       <c r="AW78" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose le seau en travers du sillon mort.
+          <t>narrateur|Amir pose le seau en travers de la trace vide.
 narrateur|L'eau s'y rassemble, fraîche.
 enfant-m|Un réservoir pour lui.
 narrateur|L'escargot gravit le bord humide, puis s'abrite.
@@ -16156,17 +16156,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Amir plante les pinces entre le creux et le banc. Un lambeau arrête les éclaboussures vers les prunes. L'eau d'un côté, le sucre de l'autre. L'escargot choisit le côté mouillé. Les pinces font la frontière. Le panier, au sec, se tait. Une prune roule sur le banc, sans tomber. Sous les pinces, la terre brille.</t>
+          <t>Amir plante les pinces entre le creux et le banc. Un bout de tissu arrête les gouttes vers les prunes. L'eau d'un côté, le sucre de l'autre. L'escargot choisit le côté mouillé. Les pinces font la frontière. Le panier, au sec, se tait. Une prune roule sur le banc, sans tomber. Sous les pinces, la terre brille.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir plante les &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt; entre le creux et le banc. Un lambeau arrête les éclaboussures vers les prunes. L'eau d'un côté, le sucre de l'autre. L'escargot choisit le côté mouillé. Les pinces font la frontière. Le panier, au sec, se tait. Une prune roule sur le banc, sans tomber. Sous les pinces, la terre brille.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir plante les &lt;emphasis level="moderate"&gt;pinces&lt;/emphasis&gt; entre le creux et le banc. Un bout de tissu arrête les gouttes vers les prunes. L'eau d'un côté, le sucre de l'autre. L'escargot choisit le côté mouillé. Les pinces font la frontière. Le panier, au sec, se tait. Une prune roule sur le banc, sans tomber. Sous les pinces, la terre brille.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Amir plante les &lt;emphasis&gt;pinces&lt;/emphasis&gt; entre le creux et le banc. Un lambeau arrête les éclaboussures vers les prunes. L'eau d'un côté, le sucre de l'autre. L'escargot choisit le côté mouillé. Les pinces font la frontière. Le panier, au sec, se tait. Une prune roule sur le banc, sans tomber. Sous les pinces, la terre brille. [pause]</t>
+          <t>Amir plante les &lt;emphasis&gt;pinces&lt;/emphasis&gt; entre le creux et le banc. Un bout de tissu arrête les gouttes vers les prunes. L'eau d'un côté, le sucre de l'autre. L'escargot choisit le côté mouillé. Les pinces font la frontière. Le panier, au sec, se tait. Une prune roule sur le banc, sans tomber. Sous les pinces, la terre brille. [pause]</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -16301,7 +16301,7 @@
       <c r="AW82" t="inlineStr">
         <is>
           <t>narrateur|Amir plante les pinces entre le creux et le banc.
-narrateur|Un lambeau arrête les éclaboussures vers les prunes.
+narrateur|Un bout de tissu arrête les gouttes vers les prunes.
 enfant-m|L'eau d'un côté, le sucre de l'autre.
 narrateur|L'escargot choisit le côté mouillé.
 papa|Les pinces font la frontière.
@@ -16524,17 +16524,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Amir tend la corde du creux jusqu'au tronc. Le lambeau fait un couloir, loin du banc. Son chemin à lui. L'escargot s'y engage, dos aux prunes. La corde l'éloigne du sucre. Le panier n'a plus à craindre l'eau. L'osier blanchit au soleil du banc. Le couloir, lui, reste sombre.</t>
+          <t>Amir tend la corde du creux jusqu'au tronc. Le bout de tissu fait un couloir, loin du banc. Son chemin à lui. L'escargot s'y engage, dos aux prunes. La corde l'éloigne du sucre. Le panier n'a plus à craindre l'eau. L'osier blanchit au soleil du banc. Le couloir, lui, reste sombre.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir tend la &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; du creux jusqu'au tronc. Le lambeau fait un couloir, loin du banc. Son chemin à lui. L'escargot s'y engage, dos aux prunes. La corde l'éloigne du sucre. Le panier n'a plus à craindre l'eau. L'osier blanchit au soleil du banc. Le couloir, lui, reste sombre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir tend la &lt;emphasis level="moderate"&gt;corde&lt;/emphasis&gt; du creux jusqu'au tronc. Le bout de tissu fait un couloir, loin du banc. Son chemin à lui. L'escargot s'y engage, dos aux prunes. La corde l'éloigne du sucre. Le panier n'a plus à craindre l'eau. L'osier blanchit au soleil du banc. Le couloir, lui, reste sombre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Amir tend la &lt;emphasis&gt;corde&lt;/emphasis&gt; du creux jusqu'au tronc. Le lambeau fait un couloir, loin du banc. Son chemin à lui. L'escargot s'y engage, dos aux prunes. La corde l'éloigne du sucre. Le panier n'a plus à craindre l'eau. L'osier blanchit au soleil du banc. Le couloir, lui, reste sombre. [pause]</t>
+          <t>Amir tend la &lt;emphasis&gt;corde&lt;/emphasis&gt; du creux jusqu'au tronc. Le bout de tissu fait un couloir, loin du banc. Son chemin à lui. L'escargot s'y engage, dos aux prunes. La corde l'éloigne du sucre. Le panier n'a plus à craindre l'eau. L'osier blanchit au soleil du banc. Le couloir, lui, reste sombre. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -16669,7 +16669,7 @@
       <c r="AW84" t="inlineStr">
         <is>
           <t>narrateur|Amir tend la corde du creux jusqu'au tronc.
-narrateur|Le lambeau fait un couloir, loin du banc.
+narrateur|Le bout de tissu fait un couloir, loin du banc.
 enfant-m|Son chemin à lui.
 narrateur|L'escargot s'y engage, dos aux prunes.
 maman|La corde l'éloigne du sucre.
@@ -16892,17 +16892,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Amir pose le seau entre le creux et les prunes. Le bleu coupe l'odeur sucrée. Deux mondes ! L'escargot entre du côté de l'eau. Le seau a choisi son camp. Les prunes aussi, sur leur banc. Une goutte chante dans le bleu. Sur le banc, une prune fendille, sans bruit.</t>
+          <t>Amir pose le seau entre le creux et les prunes. Le bleu coupe l'odeur sucrée. Deux mondes ! L'escargot entre du côté de l'eau. Le seau a choisi son camp. Les prunes aussi, sur leur banc. Une goutte chante dans le bleu. Sur le banc, une prune se fend, sans bruit.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir pose le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; entre le creux et les prunes. Le bleu coupe l'odeur sucrée. Deux mondes ! L'escargot entre du côté de l'eau. Le seau a choisi son camp. Les prunes aussi, sur leur banc. Une goutte chante dans le bleu. Sur le banc, une prune fendille, sans bruit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir pose le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; entre le creux et les prunes. Le bleu coupe l'odeur sucrée. Deux mondes ! L'escargot entre du côté de l'eau. Le seau a choisi son camp. Les prunes aussi, sur leur banc. Une goutte chante dans le bleu. Sur le banc, une prune se fend, sans bruit.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Amir pose le &lt;emphasis&gt;seau&lt;/emphasis&gt; entre le creux et les prunes. Le bleu coupe l'odeur sucrée. Deux mondes ! L'escargot entre du côté de l'eau. Le seau a choisi son camp. Les prunes aussi, sur leur banc. Une goutte chante dans le bleu. Sur le banc, une prune fendille, sans bruit. [pause]</t>
+          <t>Amir pose le &lt;emphasis&gt;seau&lt;/emphasis&gt; entre le creux et les prunes. Le bleu coupe l'odeur sucrée. Deux mondes ! L'escargot entre du côté de l'eau. Le seau a choisi son camp. Les prunes aussi, sur leur banc. Une goutte chante dans le bleu. Sur le banc, une prune se fend, sans bruit. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17043,7 +17043,7 @@
 papa|Le seau a choisi son camp.
 maman|Les prunes aussi, sur leur banc.
 narrateur|Une goutte chante dans le bleu.
-narrateur|Sur le banc, une prune fendille, sans bruit.</t>
+narrateur|Sur le banc, une prune se fend, sans bruit.</t>
         </is>
       </c>
       <c r="AX86" t="inlineStr">
@@ -17075,17 +17075,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Amir pose une main sur le seau, une autre vers le banc. Deux mondes, tu disais. Oui, il a choisi l'eau. Les prunes fendillent, sans lui. Une goutte chante dans le bleu, une dernière fois. Sous le prunier, l'abri tient, et le soleil perd.</t>
+          <t>Amir pose une main sur le seau, une autre vers le banc. Deux mondes, tu disais. Oui, il a choisi l'eau. Les prunes se fendent, sans lui. Une goutte chante dans le bleu, une dernière fois. Sous le prunier, l'abri tient, et le soleil perd.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir pose une main sur le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt;, une autre vers le banc. Deux mondes, tu disais. Oui, il a choisi l'eau. Les prunes fendillent, sans lui. Une goutte chante dans le bleu, une dernière fois. Sous le prunier, l'abri tient, et le soleil perd.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Amir pose une main sur le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt;, une autre vers le banc. Deux mondes, tu disais. Oui, il a choisi l'eau. Les prunes se fendent, sans lui. Une goutte chante dans le bleu, une dernière fois. Sous le prunier, l'abri tient, et le soleil perd.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir pose une main sur le &lt;emphasis&gt;seau&lt;/emphasis&gt;, une autre vers le banc. Deux mondes, tu disais. Oui, il a choisi l'eau. Les prunes fendillent, sans lui. Une goutte chante dans le bleu, une dernière fois. Sous le prunier, l'abri tient, et le soleil perd.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Amir pose une main sur le &lt;emphasis&gt;seau&lt;/emphasis&gt;, une autre vers le banc. Deux mondes, tu disais. Oui, il a choisi l'eau. Les prunes se fendent, sans lui. Une goutte chante dans le bleu, une dernière fois. Sous le prunier, l'abri tient, et le soleil perd.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -17226,7 +17226,7 @@
           <t>narrateur|Amir pose une main sur le seau, une autre vers le banc.
 papa|Deux mondes, tu disais.
 enfant-m|Oui, il a choisi l'eau.
-maman|Les prunes fendillent, sans lui.
+maman|Les prunes se fendent, sans lui.
 narrateur|Une goutte chante dans le bleu, une dernière fois.
 narrateur|Sous le prunier, l'abri tient, et le soleil perd.</t>
         </is>
@@ -17254,7 +17254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17311,6 +17311,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>